<commit_message>
canonical path and generate plots and tables
</commit_message>
<xml_diff>
--- a/results/meta_analysis/meta_analysis_execution_summary.xlsx
+++ b/results/meta_analysis/meta_analysis_execution_summary.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Manifest" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manifest'!$A$1:$N$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manifest'!$A$1:$R$4</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t xml:space="preserve">analysis_group</t>
   </si>
@@ -135,16 +135,25 @@
     <t xml:space="preserve">Sensitivity_RCT</t>
   </si>
   <si>
-    <t xml:space="preserve">Sensitivity RCT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SKIP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fewer than 2 studies/outcome rows; pooling not performed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensitivity evidence: use to assess robustness of the corresponding primary analysis.</t>
+    <t xml:space="preserve">Primary RCT; Sensitivity RCT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C:/Users/Jason/Projects/srma-agent-toolkit/data/processed/meta_analysis_ready/meta_analysis_ready_sensitivity_rct.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C:/Users/Jason/Projects/srma-agent-toolkit/results/meta_analysis/sensitivity_rct/forest_plot.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">analysis_set_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_composite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parent_analysis_group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source_analysis_groups</t>
   </si>
   <si>
     <t xml:space="preserve">study_count</t>
@@ -177,6 +186,15 @@
     <t xml:space="preserve">next_action</t>
   </si>
   <si>
+    <t xml:space="preserve">standalone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCT</t>
+  </si>
+  <si>
     <t xml:space="preserve">Postoperative acute kidney injury</t>
   </si>
   <si>
@@ -186,13 +204,16 @@
     <t xml:space="preserve">Mixed</t>
   </si>
   <si>
-    <t xml:space="preserve">Random-effects by default; justify fixed-effect if used</t>
+    <t xml:space="preserve">Random-effects by default; final choice belongs to the analysis stage</t>
   </si>
   <si>
     <t xml:space="preserve">NO unless explicitly prespecified and methodologically justified</t>
   </si>
   <si>
-    <t xml:space="preserve">Do not pool yet: effect measures are mixed. Harmonize or analyze separately.</t>
+    <t xml:space="preserve">Proceed to R/27 after confirming clinical compatibility.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observational</t>
   </si>
   <si>
     <t xml:space="preserve">Within 7 days after surgery; Within 7 days post-op</t>
@@ -201,22 +222,16 @@
     <t xml:space="preserve">reported_effect</t>
   </si>
   <si>
-    <t xml:space="preserve">Within 7 days after surgery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dichotomous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">raw_dichotomous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proceed to analysis-specific meta-analysis after checking clinical and methodological compatibility.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C:/Users/Jason/Projects/srma-agent-toolkit/data/processed/meta_analysis_ready/meta_analysis_ready_sensitivity_rct.csv</t>
+    <t xml:space="preserve">composite_sensitivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary_RCT + Sensitivity_RCT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Within 7 postoperative days; First 7 days postoperatively; Perioperative period (up to ~120 h postoperatively); Within 7 days after surgery</t>
   </si>
 </sst>
 </file>
@@ -546,9 +561,9 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="23.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="23.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="28.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="6.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="57.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="6.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="7.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="14.71" hidden="0" customWidth="1"/>
@@ -787,33 +802,65 @@
         <v>39</v>
       </c>
       <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4"/>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.596686774280369</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.296157008068087</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1.20218362862195</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.100681609896476</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.119180036829702</v>
+      </c>
+      <c r="O4" t="n">
+        <v>75.1220870776603</v>
+      </c>
+      <c r="P4" t="n">
+        <v>11.0398333810452</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.0115124199044159</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.162132357435773</v>
+      </c>
+      <c r="T4" t="n">
+        <v>2.19595343108578</v>
+      </c>
+      <c r="U4" t="s">
         <v>40</v>
       </c>
-      <c r="D4" t="s">
+      <c r="V4" t="s">
         <v>41</v>
       </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-      <c r="J4"/>
-      <c r="K4"/>
-      <c r="L4"/>
-      <c r="M4"/>
-      <c r="N4"/>
-      <c r="O4"/>
-      <c r="P4"/>
-      <c r="Q4"/>
-      <c r="R4"/>
-      <c r="S4"/>
-      <c r="T4"/>
-      <c r="U4"/>
-      <c r="V4"/>
       <c r="W4" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -829,19 +876,23 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="23.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="23.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="33.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="110.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="14.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="15.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="55.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="64.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="100.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="125.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="28.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="21.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="21.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="29.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="17.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="13.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="33.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="139.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="15.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="14.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="15.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="69.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="64.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="56.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="125.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -852,25 +903,25 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
-      </c>
-      <c r="I1" t="s">
-        <v>5</v>
       </c>
       <c r="J1" t="s">
         <v>49</v>
@@ -882,9 +933,21 @@
         <v>51</v>
       </c>
       <c r="M1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" t="s">
         <v>52</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>55</v>
+      </c>
+      <c r="R1" t="s">
         <v>20</v>
       </c>
     </row>
@@ -895,38 +958,50 @@
       <c r="B2" t="s">
         <v>24</v>
       </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>3</v>
+      <c r="C2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
       </c>
       <c r="E2"/>
       <c r="F2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G2" t="s">
-        <v>54</v>
-      </c>
-      <c r="H2" t="s">
-        <v>55</v>
+        <v>23</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="L2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="M2" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="N2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O2" t="s">
+        <v>62</v>
+      </c>
+      <c r="P2" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>64</v>
+      </c>
+      <c r="R2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -937,38 +1012,50 @@
       <c r="B3" t="s">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>57</v>
       </c>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="s">
+        <v>65</v>
+      </c>
+      <c r="J3" t="s">
         <v>59</v>
       </c>
-      <c r="H3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I3" t="s">
-        <v>55</v>
-      </c>
-      <c r="J3" t="s">
-        <v>60</v>
-      </c>
       <c r="K3" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="L3" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="M3" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="N3" t="s">
+        <v>67</v>
+      </c>
+      <c r="O3" t="s">
+        <v>62</v>
+      </c>
+      <c r="P3" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>64</v>
+      </c>
+      <c r="R3" t="s">
         <v>35</v>
       </c>
     </row>
@@ -979,43 +1066,57 @@
       <c r="B4" t="s">
         <v>39</v>
       </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4"/>
+      <c r="C4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
       <c r="F4" t="s">
-        <v>53</v>
-      </c>
-      <c r="G4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" t="s">
+        <v>58</v>
+      </c>
+      <c r="J4" t="s">
+        <v>59</v>
+      </c>
+      <c r="K4" t="s">
+        <v>71</v>
+      </c>
+      <c r="L4" t="s">
         <v>61</v>
       </c>
-      <c r="H4" t="s">
+      <c r="M4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O4" t="s">
         <v>62</v>
       </c>
-      <c r="I4" t="s">
+      <c r="P4" t="s">
         <v>63</v>
       </c>
-      <c r="J4" t="s">
+      <c r="Q4" t="s">
         <v>64</v>
       </c>
-      <c r="K4" t="s">
-        <v>56</v>
-      </c>
-      <c r="L4" t="s">
-        <v>57</v>
-      </c>
-      <c r="M4" t="s">
-        <v>65</v>
-      </c>
-      <c r="N4" t="s">
-        <v>66</v>
+      <c r="R4" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N4"/>
+  <autoFilter ref="A1:R4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>

</xml_diff>